<commit_message>
Fix Grist sync: blank number cells, masked failures
Grist fills empty Numeric cells with 0, so every blank capacity read as
"0 people" and failed validation. The sync now reads 0 in a Numeric
column as blank, and the fake Grist in the tests reproduces that.

The workflow step piped the sync into tee under GitHub's default shell,
which has no pipefail, so a failed sync still showed green. Run steps
now use bash explicitly.

Also: Cornerstone Makerspace's borough in the seed, and the API key's
new location in Grist (Account settings > Developer).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/find-a-venue/data/venues_master_seed.xlsx
+++ b/tools/find-a-venue/data/venues_master_seed.xlsx
@@ -2041,7 +2041,11 @@
           <t>Washington Heights</t>
         </is>
       </c>
-      <c r="G11" s="15" t="inlineStr"/>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
       <c r="H11" s="15" t="n">
         <v>40.8571</v>
       </c>

</xml_diff>

<commit_message>
Drop Grist: the Proton Sheet is the venue source again
Venue data now comes only from XLSX exports of the Proton Sheet, run
through `npm run venues:sync` and committed. The scheduled Grist sync
workflow is removed (and disabled on GitHub), along with the Grist
reader in sync.py and its test; the Grist secrets are deleted. The
README covers the Proton export flow.

The seed workbook gains dropdown lists on its fixed-value columns
(status, type, borough, precision, indoor/outdoor, cost) for when it's
imported into a new sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/find-a-venue/data/venues_master_seed.xlsx
+++ b/tools/find-a-venue/data/venues_master_seed.xlsx
@@ -3909,6 +3909,26 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="6">
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Status" error="Pick one of: Approved, Pending review, Archived" type="list">
+      <formula1>"Approved,Pending review,Archived"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Venue type" error="Pick one of: Park / public space, Privately owned public space (POPS), Library, Bar / cafe / restaurant, Club / event venue, Arts / community space, Gallery / museum, Bookstore, Church / meeting house, University, Makerspace, Community tech space, Radio station / studio, Other" type="list">
+      <formula1>"Park / public space,Privately owned public space (POPS),Library,Bar / cafe / restaurant,Club / event venue,Arts / community space,Gallery / museum,Bookstore,Church / meeting house,University,Makerspace,Community tech space,Radio station / studio,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Borough" error="Pick one of: Manhattan, Brooklyn, Queens, Bronx, Staten Island" type="list">
+      <formula1>"Manhattan,Brooklyn,Queens,Bronx,Staten Island"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Location precision" error="Pick one of: exact, approx" type="list">
+      <formula1>"exact,approx"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Indoor / outdoor" error="Pick one of: Indoor, Outdoor, Both" type="list">
+      <formula1>"Indoor,Outdoor,Both"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Cost" error="Pick one of: Free, Donation, Purchase / minimum spend, Rental fee, Ticketed by venue, Unknown" type="list">
+      <formula1>"Free,Donation,Purchase / minimum spend,Rental fee,Ticketed by venue,Unknown"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>